<commit_message>
fix bugs re senior_management, judges, eso
all tests passed
</commit_message>
<xml_diff>
--- a/refactor/source_data/FRS_liability_table.xlsx
+++ b/refactor/source_data/FRS_liability_table.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livealbany-my.sharepoint.com/personal/gchen3_albany_edu/Documents/R-projects/Florida-FRS-main_generalizable/refactor/source_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="8_{05EC5C6E-CE3D-488A-9FBB-8D386F3FD8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3239E13-A3AC-43C9-9DBE-7C1F9B5E3E88}"/>
+  <xr:revisionPtr revIDLastSave="137" documentId="8_{05EC5C6E-CE3D-488A-9FBB-8D386F3FD8B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98E543B5-2613-4CD0-B3BB-75A68769BFF4}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{B4ECBAB5-CEB2-4D8D-BCAD-5D40DFE489BD}"/>
   </bookViews>
@@ -1170,8 +1170,9 @@
     <col min="3" max="3" width="20.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1294,7 +1295,8 @@
         <v>0.91693318100993715</v>
       </c>
       <c r="G5">
-        <v>27604397</v>
+        <f>1545348000 - 1444240024</f>
+        <v>101107976</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -1344,7 +1346,8 @@
         <v>0.82832200720785465</v>
       </c>
       <c r="G7">
-        <v>101107976</v>
+        <f>138008000 - 110403603</f>
+        <v>27604397</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -1406,11 +1409,11 @@
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3">
-        <f t="shared" ref="B3:B66" ca="1" si="0">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B3" ca="1" si="0">#REF!/SUM($B$2:$B$77)</f>
         <v>1.0765145811826322E-3</v>
       </c>
       <c r="C3">
-        <f t="shared" ref="C3:C66" ca="1" si="1">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C3" ca="1" si="1">#REF!/SUM($C$2:$C$77)</f>
         <v>6.6660433036662609E-4</v>
       </c>
     </row>
@@ -1420,67 +1423,67 @@
         <v>1.0765145811826322E-3</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C67" ca="1" si="2">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C4" ca="1" si="2">#REF!/SUM($C$2:$C$77)</f>
         <v>6.6660433036662609E-4</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5">
-        <f t="shared" ref="B5:B68" ca="1" si="3">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B5" ca="1" si="3">#REF!/SUM($B$2:$B$77)</f>
         <v>1.0765145811826322E-3</v>
       </c>
       <c r="C5">
-        <f t="shared" ref="C5:C68" ca="1" si="4">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C5" ca="1" si="4">#REF!/SUM($C$2:$C$77)</f>
         <v>6.6660433036662609E-4</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6">
-        <f t="shared" ref="B6:B69" ca="1" si="5">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B6" ca="1" si="5">#REF!/SUM($B$2:$B$77)</f>
         <v>1.0765145811826322E-3</v>
       </c>
       <c r="C6">
-        <f t="shared" ref="C6:C69" ca="1" si="6">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C6" ca="1" si="6">#REF!/SUM($C$2:$C$77)</f>
         <v>6.6660433036662609E-4</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7">
-        <f t="shared" ref="B7:B70" ca="1" si="7">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B7" ca="1" si="7">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1223746433031124E-3</v>
       </c>
       <c r="C7">
-        <f t="shared" ref="C7:C70" ca="1" si="8">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C7" ca="1" si="8">#REF!/SUM($C$2:$C$77)</f>
         <v>2.6826462547526915E-3</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8">
-        <f t="shared" ref="B8:B71" ca="1" si="9">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B8" ca="1" si="9">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1223746433031124E-3</v>
       </c>
       <c r="C8">
-        <f t="shared" ref="C8:C71" ca="1" si="10">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C8" ca="1" si="10">#REF!/SUM($C$2:$C$77)</f>
         <v>2.6826462547526915E-3</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9">
-        <f t="shared" ref="B9:B72" ca="1" si="11">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B9" ca="1" si="11">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1223746433031124E-3</v>
       </c>
       <c r="C9">
-        <f t="shared" ref="C9:C72" ca="1" si="12">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C9" ca="1" si="12">#REF!/SUM($C$2:$C$77)</f>
         <v>2.6826462547526915E-3</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10">
-        <f t="shared" ref="B10:B73" ca="1" si="13">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B10" ca="1" si="13">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1223746433031124E-3</v>
       </c>
       <c r="C10">
-        <f t="shared" ref="C10:C73" ca="1" si="14">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C10" ca="1" si="14">#REF!/SUM($C$2:$C$77)</f>
         <v>2.6826462547526915E-3</v>
       </c>
     </row>
@@ -1490,667 +1493,667 @@
         <v>2.1223746433031124E-3</v>
       </c>
       <c r="C11">
-        <f t="shared" ref="C11:C74" ca="1" si="15">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C11" ca="1" si="15">#REF!/SUM($C$2:$C$77)</f>
         <v>2.6826462547526915E-3</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12">
-        <f t="shared" ref="B12:B75" ca="1" si="16">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B12" ca="1" si="16">#REF!/SUM($B$2:$B$77)</f>
         <v>7.6834650425782174E-3</v>
       </c>
       <c r="C12">
-        <f t="shared" ref="C12:C75" ca="1" si="17">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C12" ca="1" si="17">#REF!/SUM($C$2:$C$77)</f>
         <v>9.9306204145650414E-3</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13">
-        <f t="shared" ref="B13:B76" ca="1" si="18">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B13" ca="1" si="18">#REF!/SUM($B$2:$B$77)</f>
         <v>7.6834650425782174E-3</v>
       </c>
       <c r="C13">
-        <f t="shared" ref="C13:C76" ca="1" si="19">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C13" ca="1" si="19">#REF!/SUM($C$2:$C$77)</f>
         <v>9.9306204145650414E-3</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14">
-        <f t="shared" ref="B14:B77" ca="1" si="20">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B14" ca="1" si="20">#REF!/SUM($B$2:$B$77)</f>
         <v>7.6834650425782174E-3</v>
       </c>
       <c r="C14">
-        <f t="shared" ref="C14:C77" ca="1" si="21">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C14" ca="1" si="21">#REF!/SUM($C$2:$C$77)</f>
         <v>9.9306204145650414E-3</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15">
-        <f t="shared" ref="B15:B78" ca="1" si="22">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B15" ca="1" si="22">#REF!/SUM($B$2:$B$77)</f>
         <v>7.6834650425782174E-3</v>
       </c>
       <c r="C15">
-        <f t="shared" ref="C15:C78" ca="1" si="23">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C15" ca="1" si="23">#REF!/SUM($C$2:$C$77)</f>
         <v>9.9306204145650414E-3</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16">
-        <f t="shared" ref="B16:B79" ca="1" si="24">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B16" ca="1" si="24">#REF!/SUM($B$2:$B$77)</f>
         <v>7.6834650425782174E-3</v>
       </c>
       <c r="C16">
-        <f t="shared" ref="C16:C79" ca="1" si="25">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C16" ca="1" si="25">#REF!/SUM($C$2:$C$77)</f>
         <v>9.9306204145650414E-3</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17">
-        <f t="shared" ref="B17:B80" ca="1" si="26">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B17" ca="1" si="26">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1935111595973417E-2</v>
       </c>
       <c r="C17">
-        <f t="shared" ref="C17:C80" ca="1" si="27">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C17" ca="1" si="27">#REF!/SUM($C$2:$C$77)</f>
         <v>2.2839536690823743E-2</v>
       </c>
     </row>
     <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18">
-        <f t="shared" ref="B18:B81" ca="1" si="28">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B18" ca="1" si="28">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1935111595973417E-2</v>
       </c>
       <c r="C18">
-        <f t="shared" ref="C18:C81" ca="1" si="29">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C18" ca="1" si="29">#REF!/SUM($C$2:$C$77)</f>
         <v>2.2839536690823743E-2</v>
       </c>
     </row>
     <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19">
-        <f t="shared" ref="B19:B82" ca="1" si="30">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B19" ca="1" si="30">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1935111595973417E-2</v>
       </c>
       <c r="C19">
-        <f t="shared" ref="C19:C82" ca="1" si="31">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C19" ca="1" si="31">#REF!/SUM($C$2:$C$77)</f>
         <v>2.2839536690823743E-2</v>
       </c>
     </row>
     <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20">
-        <f t="shared" ref="B20:B83" ca="1" si="32">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B20" ca="1" si="32">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1935111595973417E-2</v>
       </c>
       <c r="C20">
-        <f t="shared" ref="C20:C83" ca="1" si="33">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C20" ca="1" si="33">#REF!/SUM($C$2:$C$77)</f>
         <v>2.2839536690823743E-2</v>
       </c>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21">
-        <f t="shared" ref="B21:B84" ca="1" si="34">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B21" ca="1" si="34">#REF!/SUM($B$2:$B$77)</f>
         <v>2.1935111595973417E-2</v>
       </c>
       <c r="C21">
-        <f t="shared" ref="C21:C84" ca="1" si="35">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C21" ca="1" si="35">#REF!/SUM($C$2:$C$77)</f>
         <v>2.2839536690823743E-2</v>
       </c>
     </row>
     <row r="22" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B22">
-        <f t="shared" ref="B22:B85" ca="1" si="36">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B22" ca="1" si="36">#REF!/SUM($B$2:$B$77)</f>
         <v>4.2204961524070515E-2</v>
       </c>
       <c r="C22">
-        <f t="shared" ref="C22:C85" ca="1" si="37">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C22" ca="1" si="37">#REF!/SUM($C$2:$C$77)</f>
         <v>3.9938455442621708E-2</v>
       </c>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23">
-        <f t="shared" ref="B23:B86" ca="1" si="38">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B23" ca="1" si="38">#REF!/SUM($B$2:$B$77)</f>
         <v>4.2204961524070515E-2</v>
       </c>
       <c r="C23">
-        <f t="shared" ref="C23:C86" ca="1" si="39">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C23" ca="1" si="39">#REF!/SUM($C$2:$C$77)</f>
         <v>3.9938455442621708E-2</v>
       </c>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B24">
-        <f t="shared" ref="B24:B87" ca="1" si="40">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B24" ca="1" si="40">#REF!/SUM($B$2:$B$77)</f>
         <v>4.2204961524070515E-2</v>
       </c>
       <c r="C24">
-        <f t="shared" ref="C24:C87" ca="1" si="41">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C24" ca="1" si="41">#REF!/SUM($C$2:$C$77)</f>
         <v>3.9938455442621708E-2</v>
       </c>
     </row>
     <row r="25" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B25">
-        <f t="shared" ref="B25:B88" ca="1" si="42">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B25" ca="1" si="42">#REF!/SUM($B$2:$B$77)</f>
         <v>4.2204961524070515E-2</v>
       </c>
       <c r="C25">
-        <f t="shared" ref="C25:C88" ca="1" si="43">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C25" ca="1" si="43">#REF!/SUM($C$2:$C$77)</f>
         <v>3.9938455442621708E-2</v>
       </c>
     </row>
     <row r="26" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B26">
-        <f t="shared" ref="B26:B89" ca="1" si="44">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B26" ca="1" si="44">#REF!/SUM($B$2:$B$77)</f>
         <v>4.2204961524070515E-2</v>
       </c>
       <c r="C26">
-        <f t="shared" ref="C26:C89" ca="1" si="45">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C26" ca="1" si="45">#REF!/SUM($C$2:$C$77)</f>
         <v>3.9938455442621708E-2</v>
       </c>
     </row>
     <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B27">
-        <f t="shared" ref="B27:B90" ca="1" si="46">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B27" ca="1" si="46">#REF!/SUM($B$2:$B$77)</f>
         <v>4.7984239970787997E-2</v>
       </c>
       <c r="C27">
-        <f t="shared" ref="C27:C90" ca="1" si="47">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C27" ca="1" si="47">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7839062003481453E-2</v>
       </c>
     </row>
     <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B28">
-        <f t="shared" ref="B28:B91" ca="1" si="48">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B28" ca="1" si="48">#REF!/SUM($B$2:$B$77)</f>
         <v>4.7984239970787997E-2</v>
       </c>
       <c r="C28">
-        <f t="shared" ref="C28:C91" ca="1" si="49">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C28" ca="1" si="49">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7839062003481453E-2</v>
       </c>
     </row>
     <row r="29" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B29">
-        <f t="shared" ref="B29:B92" ca="1" si="50">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B29" ca="1" si="50">#REF!/SUM($B$2:$B$77)</f>
         <v>4.7984239970787997E-2</v>
       </c>
       <c r="C29">
-        <f t="shared" ref="C29:C92" ca="1" si="51">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C29" ca="1" si="51">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7839062003481453E-2</v>
       </c>
     </row>
     <row r="30" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B30">
-        <f t="shared" ref="B30:B93" ca="1" si="52">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B30" ca="1" si="52">#REF!/SUM($B$2:$B$77)</f>
         <v>4.7984239970787997E-2</v>
       </c>
       <c r="C30">
-        <f t="shared" ref="C30:C93" ca="1" si="53">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C30" ca="1" si="53">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7839062003481453E-2</v>
       </c>
     </row>
     <row r="31" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B31">
-        <f t="shared" ref="B31:B94" ca="1" si="54">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B31" ca="1" si="54">#REF!/SUM($B$2:$B$77)</f>
         <v>4.7984239970787997E-2</v>
       </c>
       <c r="C31">
-        <f t="shared" ref="C31:C94" ca="1" si="55">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C31" ca="1" si="55">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7839062003481453E-2</v>
       </c>
     </row>
     <row r="32" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B32">
-        <f t="shared" ref="B32:B95" ca="1" si="56">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B32" ca="1" si="56">#REF!/SUM($B$2:$B$77)</f>
         <v>3.7275444377825928E-2</v>
       </c>
       <c r="C32">
-        <f t="shared" ref="C32:C95" ca="1" si="57">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C32" ca="1" si="57">#REF!/SUM($C$2:$C$77)</f>
         <v>3.7711347821865734E-2</v>
       </c>
     </row>
     <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
-        <f t="shared" ref="B33:B96" ca="1" si="58">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B33" ca="1" si="58">#REF!/SUM($B$2:$B$77)</f>
         <v>3.7275444377825928E-2</v>
       </c>
       <c r="C33">
-        <f t="shared" ref="C33:C96" ca="1" si="59">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C33" ca="1" si="59">#REF!/SUM($C$2:$C$77)</f>
         <v>3.7711347821865734E-2</v>
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
-        <f t="shared" ref="B34:B97" ca="1" si="60">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B34" ca="1" si="60">#REF!/SUM($B$2:$B$77)</f>
         <v>3.7275444377825928E-2</v>
       </c>
       <c r="C34">
-        <f t="shared" ref="C34:C97" ca="1" si="61">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C34" ca="1" si="61">#REF!/SUM($C$2:$C$77)</f>
         <v>3.7711347821865734E-2</v>
       </c>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
-        <f t="shared" ref="B35:B98" ca="1" si="62">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B35" ca="1" si="62">#REF!/SUM($B$2:$B$77)</f>
         <v>3.7275444377825928E-2</v>
       </c>
       <c r="C35">
-        <f t="shared" ref="C35:C98" ca="1" si="63">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C35" ca="1" si="63">#REF!/SUM($C$2:$C$77)</f>
         <v>3.7711347821865734E-2</v>
       </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
-        <f t="shared" ref="B36:B99" ca="1" si="64">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B36" ca="1" si="64">#REF!/SUM($B$2:$B$77)</f>
         <v>3.7275444377825928E-2</v>
       </c>
       <c r="C36">
-        <f t="shared" ref="C36:C99" ca="1" si="65">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C36" ca="1" si="65">#REF!/SUM($C$2:$C$77)</f>
         <v>3.7711347821865734E-2</v>
       </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
-        <f t="shared" ref="B37:B100" ca="1" si="66">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B37" ca="1" si="66">#REF!/SUM($B$2:$B$77)</f>
         <v>1.9858944132138987E-2</v>
       </c>
       <c r="C37">
-        <f t="shared" ref="C37:C100" ca="1" si="67">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C37" ca="1" si="67">#REF!/SUM($C$2:$C$77)</f>
         <v>1.9195863520761365E-2</v>
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
-        <f t="shared" ref="B38:B101" ca="1" si="68">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B38" ca="1" si="68">#REF!/SUM($B$2:$B$77)</f>
         <v>1.9858944132138987E-2</v>
       </c>
       <c r="C38">
-        <f t="shared" ref="C38:C101" ca="1" si="69">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C38" ca="1" si="69">#REF!/SUM($C$2:$C$77)</f>
         <v>1.9195863520761365E-2</v>
       </c>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
-        <f t="shared" ref="B39:B102" ca="1" si="70">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B39" ca="1" si="70">#REF!/SUM($B$2:$B$77)</f>
         <v>1.9858944132138987E-2</v>
       </c>
       <c r="C39">
-        <f t="shared" ref="C39:C102" ca="1" si="71">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C39" ca="1" si="71">#REF!/SUM($C$2:$C$77)</f>
         <v>1.9195863520761365E-2</v>
       </c>
     </row>
     <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
-        <f t="shared" ref="B40:B103" ca="1" si="72">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B40" ca="1" si="72">#REF!/SUM($B$2:$B$77)</f>
         <v>1.9858944132138987E-2</v>
       </c>
       <c r="C40">
-        <f t="shared" ref="C40:C103" ca="1" si="73">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C40" ca="1" si="73">#REF!/SUM($C$2:$C$77)</f>
         <v>1.9195863520761365E-2</v>
       </c>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
-        <f t="shared" ref="B41:B104" ca="1" si="74">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B41" ca="1" si="74">#REF!/SUM($B$2:$B$77)</f>
         <v>1.9858944132138987E-2</v>
       </c>
       <c r="C41">
-        <f t="shared" ref="C41:C104" ca="1" si="75">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C41" ca="1" si="75">#REF!/SUM($C$2:$C$77)</f>
         <v>1.9195863520761365E-2</v>
       </c>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
-        <f t="shared" ref="B42:B105" ca="1" si="76">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B42" ca="1" si="76">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694936E-3</v>
       </c>
       <c r="C42">
-        <f t="shared" ref="C42:C105" ca="1" si="77">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C42" ca="1" si="77">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-3</v>
       </c>
     </row>
     <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
-        <f t="shared" ref="B43:B106" ca="1" si="78">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B43" ca="1" si="78">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694936E-3</v>
       </c>
       <c r="C43">
-        <f t="shared" ref="C43:C106" ca="1" si="79">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C43" ca="1" si="79">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-3</v>
       </c>
     </row>
     <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
-        <f t="shared" ref="B44:B107" ca="1" si="80">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B44" ca="1" si="80">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694936E-3</v>
       </c>
       <c r="C44">
-        <f t="shared" ref="C44:C107" ca="1" si="81">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C44" ca="1" si="81">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-3</v>
       </c>
     </row>
     <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
-        <f t="shared" ref="B45:B108" ca="1" si="82">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B45" ca="1" si="82">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694936E-3</v>
       </c>
       <c r="C45">
-        <f t="shared" ref="C45:C108" ca="1" si="83">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C45" ca="1" si="83">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-3</v>
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
-        <f t="shared" ref="B46:B109" ca="1" si="84">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B46" ca="1" si="84">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694936E-3</v>
       </c>
       <c r="C46">
-        <f t="shared" ref="C46:C109" ca="1" si="85">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C46" ca="1" si="85">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-3</v>
       </c>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
-        <f t="shared" ref="B47:B110" ca="1" si="86">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B47" ca="1" si="86">#REF!/SUM($B$2:$B$77)</f>
         <v>4.9647360330347468E-3</v>
       </c>
       <c r="C47">
-        <f t="shared" ref="C47:C110" ca="1" si="87">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C47" ca="1" si="87">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7989658801903413E-3</v>
       </c>
     </row>
     <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
-        <f t="shared" ref="B48:B111" ca="1" si="88">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B48" ca="1" si="88">#REF!/SUM($B$2:$B$77)</f>
         <v>4.9647360330347468E-3</v>
       </c>
       <c r="C48">
-        <f t="shared" ref="C48:C111" ca="1" si="89">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C48" ca="1" si="89">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7989658801903413E-3</v>
       </c>
     </row>
     <row r="49" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B49">
-        <f t="shared" ref="B49:B112" ca="1" si="90">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B49" ca="1" si="90">#REF!/SUM($B$2:$B$77)</f>
         <v>4.9647360330347468E-3</v>
       </c>
       <c r="C49">
-        <f t="shared" ref="C49:C112" ca="1" si="91">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C49" ca="1" si="91">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7989658801903413E-3</v>
       </c>
     </row>
     <row r="50" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B50">
-        <f t="shared" ref="B50:B113" ca="1" si="92">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B50" ca="1" si="92">#REF!/SUM($B$2:$B$77)</f>
         <v>4.9647360330347468E-3</v>
       </c>
       <c r="C50">
-        <f t="shared" ref="C50:C113" ca="1" si="93">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C50" ca="1" si="93">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7989658801903413E-3</v>
       </c>
     </row>
     <row r="51" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B51">
-        <f t="shared" ref="B51:B114" ca="1" si="94">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B51" ca="1" si="94">#REF!/SUM($B$2:$B$77)</f>
         <v>4.9647360330347468E-3</v>
       </c>
       <c r="C51">
-        <f t="shared" ref="C51:C114" ca="1" si="95">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C51" ca="1" si="95">#REF!/SUM($C$2:$C$77)</f>
         <v>4.7989658801903413E-3</v>
       </c>
     </row>
     <row r="52" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B52">
-        <f t="shared" ref="B52:B115" ca="1" si="96">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B52" ca="1" si="96">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694931E-4</v>
       </c>
       <c r="C52">
-        <f t="shared" ref="C52:C115" ca="1" si="97">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C52" ca="1" si="97">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-4</v>
       </c>
     </row>
     <row r="53" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B53">
-        <f t="shared" ref="B53:B116" ca="1" si="98">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B53" ca="1" si="98">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694931E-4</v>
       </c>
       <c r="C53">
-        <f t="shared" ref="C53:C116" ca="1" si="99">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C53" ca="1" si="99">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-4</v>
       </c>
     </row>
     <row r="54" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B54">
-        <f t="shared" ref="B54:B117" ca="1" si="100">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B54" ca="1" si="100">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694931E-4</v>
       </c>
       <c r="C54">
-        <f t="shared" ref="C54:C117" ca="1" si="101">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C54" ca="1" si="101">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-4</v>
       </c>
     </row>
     <row r="55" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B55">
-        <f t="shared" ref="B55:B118" ca="1" si="102">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B55" ca="1" si="102">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694931E-4</v>
       </c>
       <c r="C55">
-        <f t="shared" ref="C55:C118" ca="1" si="103">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C55" ca="1" si="103">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-4</v>
       </c>
     </row>
     <row r="56" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B56">
-        <f t="shared" ref="B56:B119" ca="1" si="104">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B56" ca="1" si="104">#REF!/SUM($B$2:$B$77)</f>
         <v>9.9294720660694931E-4</v>
       </c>
       <c r="C56">
-        <f t="shared" ref="C56:C119" ca="1" si="105">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C56" ca="1" si="105">#REF!/SUM($C$2:$C$77)</f>
         <v>9.5979317603806825E-4</v>
       </c>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B57">
-        <f t="shared" ref="B57:B120" ca="1" si="106">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B57" ca="1" si="106">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C57">
-        <f t="shared" ref="C57:C120" ca="1" si="107">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C57" ca="1" si="107">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="58" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B58">
-        <f t="shared" ref="B58:B121" ca="1" si="108">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B58" ca="1" si="108">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C58">
-        <f t="shared" ref="C58:C121" ca="1" si="109">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C58" ca="1" si="109">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B59">
-        <f t="shared" ref="B59:B122" ca="1" si="110">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B59" ca="1" si="110">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C59">
-        <f t="shared" ref="C59:C122" ca="1" si="111">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C59" ca="1" si="111">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B60">
-        <f t="shared" ref="B60:B123" ca="1" si="112">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B60" ca="1" si="112">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C60">
-        <f t="shared" ref="C60:C123" ca="1" si="113">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C60" ca="1" si="113">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="61" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B61">
-        <f t="shared" ref="B61:B124" ca="1" si="114">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B61" ca="1" si="114">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C61">
-        <f t="shared" ref="C61:C124" ca="1" si="115">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C61" ca="1" si="115">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="62" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B62">
-        <f t="shared" ref="B62:B125" ca="1" si="116">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B62" ca="1" si="116">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C62">
-        <f t="shared" ref="C62:C125" ca="1" si="117">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C62" ca="1" si="117">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="63" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B63">
-        <f t="shared" ref="B63:B126" ca="1" si="118">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B63" ca="1" si="118">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C63">
-        <f t="shared" ref="C63:C126" ca="1" si="119">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C63" ca="1" si="119">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="64" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B64">
-        <f t="shared" ref="B64:B127" ca="1" si="120">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B64" ca="1" si="120">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C64">
-        <f t="shared" ref="C64:C127" ca="1" si="121">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C64" ca="1" si="121">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="65" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B65">
-        <f t="shared" ref="B65:B128" ca="1" si="122">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B65" ca="1" si="122">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C65">
-        <f t="shared" ref="C65:C128" ca="1" si="123">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C65" ca="1" si="123">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="66" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B66">
-        <f t="shared" ref="B66:B129" ca="1" si="124">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B66" ca="1" si="124">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C66">
-        <f t="shared" ref="C66:C129" ca="1" si="125">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C66" ca="1" si="125">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="67" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B67">
-        <f t="shared" ref="B67:B77" ca="1" si="126">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B67" ca="1" si="126">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C67">
-        <f t="shared" ref="C67:C77" ca="1" si="127">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C67" ca="1" si="127">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="68" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B68">
-        <f t="shared" ref="B68:B78" ca="1" si="128">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B68" ca="1" si="128">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C68">
-        <f t="shared" ref="C68:C78" ca="1" si="129">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C68" ca="1" si="129">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="69" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B69">
-        <f t="shared" ref="B69:B79" ca="1" si="130">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B69" ca="1" si="130">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C69">
-        <f t="shared" ref="C69:C79" ca="1" si="131">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C69" ca="1" si="131">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="70" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B70">
-        <f t="shared" ref="B70:B80" ca="1" si="132">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B70" ca="1" si="132">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C70">
-        <f t="shared" ref="C70:C80" ca="1" si="133">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C70" ca="1" si="133">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="71" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B71">
-        <f t="shared" ref="B71:B81" ca="1" si="134">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B71" ca="1" si="134">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C71">
-        <f t="shared" ref="C71:C81" ca="1" si="135">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C71" ca="1" si="135">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="72" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B72">
-        <f t="shared" ref="B72:B82" ca="1" si="136">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B72" ca="1" si="136">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C72">
-        <f t="shared" ref="C72:C82" ca="1" si="137">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C72" ca="1" si="137">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="73" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B73">
-        <f t="shared" ref="B73:B83" ca="1" si="138">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B73" ca="1" si="138">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C73">
-        <f t="shared" ref="C73:C83" ca="1" si="139">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C73" ca="1" si="139">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="74" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B74">
-        <f t="shared" ref="B74:B84" ca="1" si="140">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B74" ca="1" si="140">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C74">
-        <f t="shared" ref="C74:C84" ca="1" si="141">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C74" ca="1" si="141">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="75" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B75">
-        <f t="shared" ref="B75:B85" ca="1" si="142">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B75" ca="1" si="142">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C75">
-        <f t="shared" ref="C75:C85" ca="1" si="143">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C75" ca="1" si="143">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="76" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B76">
-        <f t="shared" ref="B76:B86" ca="1" si="144">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B76" ca="1" si="144">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C76">
-        <f t="shared" ref="C76:C86" ca="1" si="145">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C76" ca="1" si="145">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>
     <row r="77" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B77">
-        <f t="shared" ref="B77:B87" ca="1" si="146">#REF!/SUM($B$2:$B$77)</f>
+        <f t="shared" ref="B77" ca="1" si="146">#REF!/SUM($B$2:$B$77)</f>
         <v>9.4566400629233593E-4</v>
       </c>
       <c r="C77">
-        <f t="shared" ref="C77:C87" ca="1" si="147">#REF!/SUM($C$2:$C$77)</f>
+        <f t="shared" ref="C77" ca="1" si="147">#REF!/SUM($C$2:$C$77)</f>
         <v>9.1408873908387458E-4</v>
       </c>
     </row>

</xml_diff>